<commit_message>
fix(inventory): publish lại sau khi sửa giá phải đồng bộ giá cho chỗ chưa bán
Sửa giá hạng vé chỉ làm được khi sự kiện đã rút xuống (EditableEvent), rồi publish lại. Publish lại gửi
session.published với giá mới nhưng JdbcSessionMaterializer chỉ đồng bộ cửa bán, trần mua vé và toạ độ,
không đồng bộ giá: Catalog niêm yết một giá, Inventory — nguồn giá của đơn — giữ giá cũ vĩnh viễn. Phát
hiện qua k6: "Sát sàn 16 · Courtside" niêm yết 25.000đ nhưng đơn tính 2.500.000đ.

syncUnsoldPrices cập nhật giá và tên hạng vé cho chỗ chưa có ai đụng tới (AVAILABLE, BLOCKED, kể cả đơn vị
ảo của vé đứng). Chỗ đã bán / đang giữ / đã đặt giữ giá khách đã thấy, đúng mối lo của bản trước. Sự kiện
đã lệch sẵn được chữa bằng POST .../resync-inventory.

Test: MaterializeSessionIT.publish_lai_thi_dong_bo_gia_cho_chua_ban (đỏ khi bỏ bản sửa, xanh khi có).
</commit_message>
<xml_diff>
--- a/docs/testing/danh-muc-test/backend-catalog-service.xlsx
+++ b/docs/testing/danh-muc-test/backend-catalog-service.xlsx
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="H6" s="5" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="7">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="H7" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="8">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="H8" s="5" t="n">
-        <v>0.026</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="9">
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="H9" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="10">
@@ -814,7 +814,7 @@
         </is>
       </c>
       <c r="H11" s="5" t="n">
-        <v>0.027</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="12">
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="13">
@@ -890,7 +890,7 @@
         </is>
       </c>
       <c r="H13" s="5" t="n">
-        <v>0</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="14">
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="H14" s="5" t="n">
-        <v>0.011</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="15">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="H15" s="5" t="n">
-        <v>0.016</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="16">
@@ -1004,7 +1004,7 @@
         </is>
       </c>
       <c r="H16" s="5" t="n">
-        <v>0.178</v>
+        <v>0.09</v>
       </c>
     </row>
     <row r="17">
@@ -1042,7 +1042,7 @@
         </is>
       </c>
       <c r="H17" s="5" t="n">
-        <v>0.006</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="18">
@@ -1080,7 +1080,7 @@
         </is>
       </c>
       <c r="H18" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="19">
@@ -1118,7 +1118,7 @@
         </is>
       </c>
       <c r="H19" s="5" t="n">
-        <v>0.06</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="20">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="H20" s="5" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="21">
@@ -1194,7 +1194,7 @@
         </is>
       </c>
       <c r="H21" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="22">
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="H22" s="5" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="23">
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="H23" s="5" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="24">
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="H24" s="5" t="n">
-        <v>0.011</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="25">
@@ -1346,7 +1346,7 @@
         </is>
       </c>
       <c r="H25" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="26">
@@ -1384,7 +1384,7 @@
         </is>
       </c>
       <c r="H26" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="27">
@@ -1422,7 +1422,7 @@
         </is>
       </c>
       <c r="H27" s="5" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="28">
@@ -1460,7 +1460,7 @@
         </is>
       </c>
       <c r="H28" s="5" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="29">
@@ -1498,7 +1498,7 @@
         </is>
       </c>
       <c r="H29" s="5" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="30">
@@ -1536,7 +1536,7 @@
         </is>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="31">
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="H31" s="5" t="n">
-        <v>2.592</v>
+        <v>2.049</v>
       </c>
     </row>
     <row r="32">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="H32" s="5" t="n">
-        <v>0.019</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="33">
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="H33" s="5" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="34">
@@ -1688,7 +1688,7 @@
         </is>
       </c>
       <c r="H34" s="5" t="n">
-        <v>0.045</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="35">
@@ -1764,7 +1764,7 @@
         </is>
       </c>
       <c r="H36" s="5" t="n">
-        <v>0.011</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="37">
@@ -1802,7 +1802,7 @@
         </is>
       </c>
       <c r="H37" s="5" t="n">
-        <v>0.011</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="38">
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="H38" s="5" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="39">
@@ -1878,7 +1878,7 @@
         </is>
       </c>
       <c r="H39" s="5" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="40">
@@ -1916,7 +1916,7 @@
         </is>
       </c>
       <c r="H40" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="41">
@@ -1992,7 +1992,7 @@
         </is>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.011</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="43">
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="H43" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="44">
@@ -2068,7 +2068,7 @@
         </is>
       </c>
       <c r="H44" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="45">
@@ -2106,7 +2106,7 @@
         </is>
       </c>
       <c r="H45" s="5" t="n">
-        <v>0.016</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="46">
@@ -2144,7 +2144,7 @@
         </is>
       </c>
       <c r="H46" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="47">
@@ -2182,7 +2182,7 @@
         </is>
       </c>
       <c r="H47" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="48">
@@ -2220,7 +2220,7 @@
         </is>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="49">
@@ -2258,7 +2258,7 @@
         </is>
       </c>
       <c r="H49" s="5" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="50">
@@ -2296,7 +2296,7 @@
         </is>
       </c>
       <c r="H50" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="51">
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="H51" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="52">
@@ -2372,7 +2372,7 @@
         </is>
       </c>
       <c r="H52" s="5" t="n">
-        <v>0.013</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="53">
@@ -2410,7 +2410,7 @@
         </is>
       </c>
       <c r="H53" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="54">
@@ -2486,7 +2486,7 @@
         </is>
       </c>
       <c r="H55" s="5" t="n">
-        <v>0.004</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="56">
@@ -2524,7 +2524,7 @@
         </is>
       </c>
       <c r="H56" s="5" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="57">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="H57" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="58">
@@ -2638,7 +2638,7 @@
         </is>
       </c>
       <c r="H59" s="5" t="n">
-        <v>0.139</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="60">
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="H60" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="61">
@@ -2714,7 +2714,7 @@
         </is>
       </c>
       <c r="H61" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="62">
@@ -2752,7 +2752,7 @@
         </is>
       </c>
       <c r="H62" s="5" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="63">
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="H63" s="5" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="64">
@@ -2828,7 +2828,7 @@
         </is>
       </c>
       <c r="H64" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="65">
@@ -2866,7 +2866,7 @@
         </is>
       </c>
       <c r="H65" s="5" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="66">
@@ -2904,7 +2904,7 @@
         </is>
       </c>
       <c r="H66" s="5" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="67">
@@ -2942,7 +2942,7 @@
         </is>
       </c>
       <c r="H67" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="68">
@@ -2980,7 +2980,7 @@
         </is>
       </c>
       <c r="H68" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="69">
@@ -3018,7 +3018,7 @@
         </is>
       </c>
       <c r="H69" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="70">
@@ -3056,7 +3056,7 @@
         </is>
       </c>
       <c r="H70" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="71">
@@ -3094,7 +3094,7 @@
         </is>
       </c>
       <c r="H71" s="5" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="72">
@@ -3132,7 +3132,7 @@
         </is>
       </c>
       <c r="H72" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="73">
@@ -3170,7 +3170,7 @@
         </is>
       </c>
       <c r="H73" s="5" t="n">
-        <v>0.006</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="74">
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="H74" s="5" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="75">
@@ -3246,7 +3246,7 @@
         </is>
       </c>
       <c r="H75" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="76">
@@ -3284,7 +3284,7 @@
         </is>
       </c>
       <c r="H76" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="77">
@@ -3322,7 +3322,7 @@
         </is>
       </c>
       <c r="H77" s="5" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="78">
@@ -3360,7 +3360,7 @@
         </is>
       </c>
       <c r="H78" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="79">
@@ -3398,7 +3398,7 @@
         </is>
       </c>
       <c r="H79" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="80">
@@ -3436,7 +3436,7 @@
         </is>
       </c>
       <c r="H80" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="81">
@@ -3474,7 +3474,7 @@
         </is>
       </c>
       <c r="H81" s="5" t="n">
-        <v>0.013</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="82">
@@ -3550,7 +3550,7 @@
         </is>
       </c>
       <c r="H83" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="84">
@@ -3626,7 +3626,7 @@
         </is>
       </c>
       <c r="H85" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="86">
@@ -3664,7 +3664,7 @@
         </is>
       </c>
       <c r="H86" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="87">
@@ -3702,7 +3702,7 @@
         </is>
       </c>
       <c r="H87" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="88">
@@ -3778,7 +3778,7 @@
         </is>
       </c>
       <c r="H89" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="90">
@@ -3816,7 +3816,7 @@
         </is>
       </c>
       <c r="H90" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="91">
@@ -3854,7 +3854,7 @@
         </is>
       </c>
       <c r="H91" s="5" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="92">
@@ -3888,7 +3888,7 @@
         </is>
       </c>
       <c r="H92" s="5" t="n">
-        <v>0.01</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="93">
@@ -3922,7 +3922,7 @@
         </is>
       </c>
       <c r="H93" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="94">
@@ -3956,7 +3956,7 @@
         </is>
       </c>
       <c r="H94" s="5" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="95">
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="H95" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="96">
@@ -4024,7 +4024,7 @@
         </is>
       </c>
       <c r="H96" s="5" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="97">
@@ -4096,7 +4096,7 @@
         </is>
       </c>
       <c r="H98" s="5" t="n">
-        <v>0.063</v>
+        <v>0.056</v>
       </c>
     </row>
     <row r="99">
@@ -4134,7 +4134,7 @@
         </is>
       </c>
       <c r="H99" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="100">
@@ -4172,7 +4172,7 @@
         </is>
       </c>
       <c r="H100" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="101">
@@ -4210,7 +4210,7 @@
         </is>
       </c>
       <c r="H101" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="102">
@@ -4248,7 +4248,7 @@
         </is>
       </c>
       <c r="H102" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="103">
@@ -4286,7 +4286,7 @@
         </is>
       </c>
       <c r="H103" s="5" t="n">
-        <v>0.013</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="104">
@@ -4362,7 +4362,7 @@
         </is>
       </c>
       <c r="H105" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="106">
@@ -4400,7 +4400,7 @@
         </is>
       </c>
       <c r="H106" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="107">
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="H107" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="108">
@@ -4476,7 +4476,7 @@
         </is>
       </c>
       <c r="H108" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="109">
@@ -4552,7 +4552,7 @@
         </is>
       </c>
       <c r="H110" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="111">
@@ -4590,7 +4590,7 @@
         </is>
       </c>
       <c r="H111" s="5" t="n">
-        <v>0.008</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="112">
@@ -4666,7 +4666,7 @@
         </is>
       </c>
       <c r="H113" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="114">
@@ -4704,7 +4704,7 @@
         </is>
       </c>
       <c r="H114" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="115">
@@ -4742,7 +4742,7 @@
         </is>
       </c>
       <c r="H115" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="116">
@@ -4780,7 +4780,7 @@
         </is>
       </c>
       <c r="H116" s="5" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="117">
@@ -4818,7 +4818,7 @@
         </is>
       </c>
       <c r="H117" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="118">
@@ -4894,7 +4894,7 @@
         </is>
       </c>
       <c r="H119" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="120">
@@ -4932,7 +4932,7 @@
         </is>
       </c>
       <c r="H120" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="121">
@@ -4970,7 +4970,7 @@
         </is>
       </c>
       <c r="H121" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="122">
@@ -5008,7 +5008,7 @@
         </is>
       </c>
       <c r="H122" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="123">
@@ -5122,7 +5122,7 @@
         </is>
       </c>
       <c r="H125" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="126">
@@ -5160,7 +5160,7 @@
         </is>
       </c>
       <c r="H126" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="127">
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="H127" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="128">
@@ -5228,7 +5228,7 @@
         </is>
       </c>
       <c r="H128" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="129">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="H129" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="130">
@@ -5296,7 +5296,7 @@
         </is>
       </c>
       <c r="H130" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="131">
@@ -5330,7 +5330,7 @@
         </is>
       </c>
       <c r="H131" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="132">
@@ -5364,7 +5364,7 @@
         </is>
       </c>
       <c r="H132" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="133">
@@ -5466,7 +5466,7 @@
         </is>
       </c>
       <c r="H135" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="136">
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="H136" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="137">
@@ -5534,7 +5534,7 @@
         </is>
       </c>
       <c r="H137" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="138">
@@ -5572,7 +5572,7 @@
         </is>
       </c>
       <c r="H138" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="139">
@@ -5610,7 +5610,7 @@
         </is>
       </c>
       <c r="H139" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="140">
@@ -5648,7 +5648,7 @@
         </is>
       </c>
       <c r="H140" s="5" t="n">
-        <v>0.021</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="141">
@@ -5686,7 +5686,7 @@
         </is>
       </c>
       <c r="H141" s="5" t="n">
-        <v>0.02</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="142">
@@ -5724,7 +5724,7 @@
         </is>
       </c>
       <c r="H142" s="5" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="143">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="H143" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="144">
@@ -5800,7 +5800,7 @@
         </is>
       </c>
       <c r="H144" s="5" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="145">
@@ -5838,7 +5838,7 @@
         </is>
       </c>
       <c r="H145" s="5" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="146">
@@ -5876,7 +5876,7 @@
         </is>
       </c>
       <c r="H146" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="147">
@@ -5914,7 +5914,7 @@
         </is>
       </c>
       <c r="H147" s="5" t="n">
-        <v>0.177</v>
+        <v>0.179</v>
       </c>
     </row>
     <row r="148">
@@ -5952,7 +5952,7 @@
         </is>
       </c>
       <c r="H148" s="5" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="149">
@@ -5990,7 +5990,7 @@
         </is>
       </c>
       <c r="H149" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="150">
@@ -6028,7 +6028,7 @@
         </is>
       </c>
       <c r="H150" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="151">
@@ -6066,7 +6066,7 @@
         </is>
       </c>
       <c r="H151" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="152">
@@ -6104,7 +6104,7 @@
         </is>
       </c>
       <c r="H152" s="5" t="n">
-        <v>0.007</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="153">
@@ -6142,7 +6142,7 @@
         </is>
       </c>
       <c r="H153" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="154">
@@ -6294,7 +6294,7 @@
         </is>
       </c>
       <c r="H157" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="158">
@@ -6370,7 +6370,7 @@
         </is>
       </c>
       <c r="H159" s="5" t="n">
-        <v>0.001</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="160">
@@ -6404,7 +6404,7 @@
         </is>
       </c>
       <c r="H160" s="5" t="n">
-        <v>0.006</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="161">
@@ -6438,7 +6438,7 @@
         </is>
       </c>
       <c r="H161" s="5" t="n">
-        <v>0.01</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="162">
@@ -6472,7 +6472,7 @@
         </is>
       </c>
       <c r="H162" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="163">
@@ -6506,7 +6506,7 @@
         </is>
       </c>
       <c r="H163" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="164">
@@ -6540,7 +6540,7 @@
         </is>
       </c>
       <c r="H164" s="5" t="n">
-        <v>0.007</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="165">
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="H165" s="5" t="n">
-        <v>0.147</v>
+        <v>0.139</v>
       </c>
     </row>
     <row r="166">
@@ -6608,7 +6608,7 @@
         </is>
       </c>
       <c r="H166" s="5" t="n">
-        <v>0.01</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="167">
@@ -6642,7 +6642,7 @@
         </is>
       </c>
       <c r="H167" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="168">
@@ -6676,7 +6676,7 @@
         </is>
       </c>
       <c r="H168" s="5" t="n">
-        <v>4.413</v>
+        <v>3.705</v>
       </c>
     </row>
     <row r="169">
@@ -6710,7 +6710,7 @@
         </is>
       </c>
       <c r="H169" s="5" t="n">
-        <v>0.68</v>
+        <v>0.424</v>
       </c>
     </row>
     <row r="170">
@@ -6744,7 +6744,7 @@
         </is>
       </c>
       <c r="H170" s="5" t="n">
-        <v>0.066</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="171">
@@ -6778,7 +6778,7 @@
         </is>
       </c>
       <c r="H171" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="172">
@@ -6812,7 +6812,7 @@
         </is>
       </c>
       <c r="H172" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="173">
@@ -6846,7 +6846,7 @@
         </is>
       </c>
       <c r="H173" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="174">
@@ -6880,7 +6880,7 @@
         </is>
       </c>
       <c r="H174" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="175">
@@ -6914,7 +6914,7 @@
         </is>
       </c>
       <c r="H175" s="5" t="n">
-        <v>0.005</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="176">
@@ -7016,7 +7016,7 @@
         </is>
       </c>
       <c r="H178" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="179">
@@ -7130,7 +7130,7 @@
         </is>
       </c>
       <c r="H181" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="182">
@@ -7168,7 +7168,7 @@
         </is>
       </c>
       <c r="H182" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="183">
@@ -7244,7 +7244,7 @@
         </is>
       </c>
       <c r="H184" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="185">
@@ -7320,7 +7320,7 @@
         </is>
       </c>
       <c r="H186" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="187">
@@ -7358,7 +7358,7 @@
         </is>
       </c>
       <c r="H187" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="188">
@@ -7396,7 +7396,7 @@
         </is>
       </c>
       <c r="H188" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="189">
@@ -7510,7 +7510,7 @@
         </is>
       </c>
       <c r="H191" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="192">
@@ -7586,7 +7586,7 @@
         </is>
       </c>
       <c r="H193" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="194">
@@ -7624,7 +7624,7 @@
         </is>
       </c>
       <c r="H194" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="195">
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="H195" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="196">
@@ -7700,7 +7700,7 @@
         </is>
       </c>
       <c r="H196" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="197">
@@ -7738,7 +7738,7 @@
         </is>
       </c>
       <c r="H197" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="198">
@@ -7776,7 +7776,7 @@
         </is>
       </c>
       <c r="H198" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="199">
@@ -7814,7 +7814,7 @@
         </is>
       </c>
       <c r="H199" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="200">
@@ -7852,7 +7852,7 @@
         </is>
       </c>
       <c r="H200" s="5" t="n">
-        <v>0.005</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="201">
@@ -7890,7 +7890,7 @@
         </is>
       </c>
       <c r="H201" s="5" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="202">
@@ -7966,7 +7966,7 @@
         </is>
       </c>
       <c r="H203" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="204">
@@ -8004,7 +8004,7 @@
         </is>
       </c>
       <c r="H204" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="205">
@@ -8042,7 +8042,7 @@
         </is>
       </c>
       <c r="H205" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="206">
@@ -8232,7 +8232,7 @@
         </is>
       </c>
       <c r="H210" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211">
@@ -8270,7 +8270,7 @@
         </is>
       </c>
       <c r="H211" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="212">
@@ -8346,7 +8346,7 @@
         </is>
       </c>
       <c r="H213" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -8384,7 +8384,7 @@
         </is>
       </c>
       <c r="H214" s="5" t="n">
-        <v>0.002</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="215">
@@ -8498,7 +8498,7 @@
         </is>
       </c>
       <c r="H217" s="5" t="n">
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="218">
@@ -8536,7 +8536,7 @@
         </is>
       </c>
       <c r="H218" s="5" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="219">
@@ -8574,7 +8574,7 @@
         </is>
       </c>
       <c r="H219" s="5" t="n">
-        <v>0.011</v>
+        <v>0</v>
       </c>
     </row>
     <row r="220">
@@ -8650,7 +8650,7 @@
         </is>
       </c>
       <c r="H221" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="222">
@@ -8764,7 +8764,7 @@
         </is>
       </c>
       <c r="H224" s="5" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="225">
@@ -8836,7 +8836,7 @@
         </is>
       </c>
       <c r="H226" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="227">
@@ -8870,7 +8870,7 @@
         </is>
       </c>
       <c r="H227" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="228">
@@ -8904,7 +8904,7 @@
         </is>
       </c>
       <c r="H228" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="229">
@@ -8938,7 +8938,7 @@
         </is>
       </c>
       <c r="H229" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="230">
@@ -8972,7 +8972,7 @@
         </is>
       </c>
       <c r="H230" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="231">
@@ -9006,7 +9006,7 @@
         </is>
       </c>
       <c r="H231" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="232">
@@ -9040,7 +9040,7 @@
         </is>
       </c>
       <c r="H232" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="233">
@@ -9074,7 +9074,7 @@
         </is>
       </c>
       <c r="H233" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="234">
@@ -9244,7 +9244,7 @@
         </is>
       </c>
       <c r="H238" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="239">
@@ -9278,7 +9278,7 @@
         </is>
       </c>
       <c r="H239" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="240">
@@ -9312,7 +9312,7 @@
         </is>
       </c>
       <c r="H240" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="241">
@@ -9346,7 +9346,7 @@
         </is>
       </c>
       <c r="H241" s="5" t="n">
-        <v>0.005</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="242">
@@ -9414,7 +9414,7 @@
         </is>
       </c>
       <c r="H243" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="244">
@@ -9448,7 +9448,7 @@
         </is>
       </c>
       <c r="H244" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="245">
@@ -9482,7 +9482,7 @@
         </is>
       </c>
       <c r="H245" s="5" t="n">
-        <v>0</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="246">
@@ -9516,7 +9516,7 @@
         </is>
       </c>
       <c r="H246" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="247">
@@ -9550,7 +9550,7 @@
         </is>
       </c>
       <c r="H247" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="248">
@@ -9584,7 +9584,7 @@
         </is>
       </c>
       <c r="H248" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="249">
@@ -9698,7 +9698,7 @@
         </is>
       </c>
       <c r="H251" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="252">
@@ -9736,7 +9736,7 @@
         </is>
       </c>
       <c r="H252" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="253">
@@ -9774,7 +9774,7 @@
         </is>
       </c>
       <c r="H253" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="254">
@@ -9812,7 +9812,7 @@
         </is>
       </c>
       <c r="H254" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="255">
@@ -9850,7 +9850,7 @@
         </is>
       </c>
       <c r="H255" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="256">
@@ -9888,7 +9888,7 @@
         </is>
       </c>
       <c r="H256" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="257">
@@ -9926,7 +9926,7 @@
         </is>
       </c>
       <c r="H257" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="258">
@@ -10002,7 +10002,7 @@
         </is>
       </c>
       <c r="H259" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="260">
@@ -10078,7 +10078,7 @@
         </is>
       </c>
       <c r="H261" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="262">
@@ -10116,7 +10116,7 @@
         </is>
       </c>
       <c r="H262" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="263">
@@ -10154,7 +10154,7 @@
         </is>
       </c>
       <c r="H263" s="5" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="264">
@@ -10192,7 +10192,7 @@
         </is>
       </c>
       <c r="H264" s="5" t="n">
-        <v>0.005</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="265">
@@ -10230,7 +10230,7 @@
         </is>
       </c>
       <c r="H265" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="266">
@@ -10268,7 +10268,7 @@
         </is>
       </c>
       <c r="H266" s="5" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="267">
@@ -10306,7 +10306,7 @@
         </is>
       </c>
       <c r="H267" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="268">
@@ -10340,7 +10340,7 @@
         </is>
       </c>
       <c r="H268" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="269">
@@ -10374,7 +10374,7 @@
         </is>
       </c>
       <c r="H269" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="270">
@@ -10544,7 +10544,7 @@
         </is>
       </c>
       <c r="H274" s="5" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="275">
@@ -10612,7 +10612,7 @@
         </is>
       </c>
       <c r="H276" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="277">
@@ -10646,7 +10646,7 @@
         </is>
       </c>
       <c r="H277" s="5" t="n">
-        <v>0.007</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="278">
@@ -10680,7 +10680,7 @@
         </is>
       </c>
       <c r="H278" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="279">
@@ -10714,7 +10714,7 @@
         </is>
       </c>
       <c r="H279" s="5" t="n">
-        <v>0.006</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="280">
@@ -10748,7 +10748,7 @@
         </is>
       </c>
       <c r="H280" s="5" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="281">
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="H281" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="282">
@@ -10850,7 +10850,7 @@
         </is>
       </c>
       <c r="H283" s="5" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="284">
@@ -10884,7 +10884,7 @@
         </is>
       </c>
       <c r="H284" s="5" t="n">
-        <v>0.003</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="285">
@@ -10918,7 +10918,7 @@
         </is>
       </c>
       <c r="H285" s="5" t="n">
-        <v>0.001</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="286">
@@ -10952,7 +10952,7 @@
         </is>
       </c>
       <c r="H286" s="5" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="287">
@@ -10986,7 +10986,7 @@
         </is>
       </c>
       <c r="H287" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="288">
@@ -11020,7 +11020,7 @@
         </is>
       </c>
       <c r="H288" s="5" t="n">
-        <v>0.052</v>
+        <v>0.047</v>
       </c>
     </row>
     <row r="289">
@@ -11054,7 +11054,7 @@
         </is>
       </c>
       <c r="H289" s="5" t="n">
-        <v>0.006</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="290">
@@ -11088,7 +11088,7 @@
         </is>
       </c>
       <c r="H290" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="291">
@@ -11122,7 +11122,7 @@
         </is>
       </c>
       <c r="H291" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="292">
@@ -11190,7 +11190,7 @@
         </is>
       </c>
       <c r="H293" s="5" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="294">
@@ -11224,7 +11224,7 @@
         </is>
       </c>
       <c r="H294" s="5" t="n">
-        <v>0.008</v>
+        <v>0</v>
       </c>
     </row>
     <row r="295">
@@ -11292,7 +11292,7 @@
         </is>
       </c>
       <c r="H296" s="5" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
     </row>
     <row r="297">
@@ -11326,7 +11326,7 @@
         </is>
       </c>
       <c r="H297" s="5" t="n">
-        <v>0.004</v>
+        <v>0.002</v>
       </c>
     </row>
     <row r="298">
@@ -11364,7 +11364,7 @@
         </is>
       </c>
       <c r="H298" s="5" t="n">
-        <v>0.024</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="299">
@@ -11402,7 +11402,7 @@
         </is>
       </c>
       <c r="H299" s="5" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="300">
@@ -11478,7 +11478,7 @@
         </is>
       </c>
       <c r="H301" s="5" t="n">
-        <v>0.011</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="302">
@@ -11516,7 +11516,7 @@
         </is>
       </c>
       <c r="H302" s="5" t="n">
-        <v>0.01</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="303">
@@ -11554,7 +11554,7 @@
         </is>
       </c>
       <c r="H303" s="5" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="304">
@@ -11592,7 +11592,7 @@
         </is>
       </c>
       <c r="H304" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="305">
@@ -11630,7 +11630,7 @@
         </is>
       </c>
       <c r="H305" s="5" t="n">
-        <v>0.029</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="306">
@@ -11668,7 +11668,7 @@
         </is>
       </c>
       <c r="H306" s="5" t="n">
-        <v>0.006</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="307">
@@ -11706,7 +11706,7 @@
         </is>
       </c>
       <c r="H307" s="5" t="n">
-        <v>0</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="308">
@@ -11744,7 +11744,7 @@
         </is>
       </c>
       <c r="H308" s="5" t="n">
-        <v>0.003</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="309">
@@ -11782,7 +11782,7 @@
         </is>
       </c>
       <c r="H309" s="5" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="310">
@@ -11820,7 +11820,7 @@
         </is>
       </c>
       <c r="H310" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="311">
@@ -11896,7 +11896,7 @@
         </is>
       </c>
       <c r="H312" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="313">
@@ -11934,7 +11934,7 @@
         </is>
       </c>
       <c r="H313" s="5" t="n">
-        <v>0.025</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="314">
@@ -11972,7 +11972,7 @@
         </is>
       </c>
       <c r="H314" s="5" t="n">
-        <v>0.012</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="315">
@@ -12048,7 +12048,7 @@
         </is>
       </c>
       <c r="H316" s="5" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="317">
@@ -12086,7 +12086,7 @@
         </is>
       </c>
       <c r="H317" s="5" t="n">
-        <v>0.391</v>
+        <v>0.336</v>
       </c>
     </row>
     <row r="318">
@@ -12124,7 +12124,7 @@
         </is>
       </c>
       <c r="H318" s="5" t="n">
-        <v>0.093</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="319">
@@ -12238,7 +12238,7 @@
         </is>
       </c>
       <c r="H321" s="5" t="n">
-        <v>0.019</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="322">
@@ -12276,7 +12276,7 @@
         </is>
       </c>
       <c r="H322" s="5" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="323">
@@ -12314,7 +12314,7 @@
         </is>
       </c>
       <c r="H323" s="5" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="324">
@@ -12352,7 +12352,7 @@
         </is>
       </c>
       <c r="H324" s="5" t="n">
-        <v>0.011</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="325">
@@ -12390,7 +12390,7 @@
         </is>
       </c>
       <c r="H325" s="5" t="n">
-        <v>0.045</v>
+        <v>0.046</v>
       </c>
     </row>
     <row r="326">
@@ -12466,7 +12466,7 @@
         </is>
       </c>
       <c r="H327" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="328">
@@ -12504,7 +12504,7 @@
         </is>
       </c>
       <c r="H328" s="5" t="n">
-        <v>0.004</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="329">
@@ -12580,7 +12580,7 @@
         </is>
       </c>
       <c r="H330" s="5" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="331">
@@ -12618,7 +12618,7 @@
         </is>
       </c>
       <c r="H331" s="5" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="332">
@@ -12656,7 +12656,7 @@
         </is>
       </c>
       <c r="H332" s="5" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="333">
@@ -12694,7 +12694,7 @@
         </is>
       </c>
       <c r="H333" s="5" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="334">
@@ -12732,7 +12732,7 @@
         </is>
       </c>
       <c r="H334" s="5" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="335">
@@ -12770,7 +12770,7 @@
         </is>
       </c>
       <c r="H335" s="5" t="n">
-        <v>0.01</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="336">
@@ -12808,7 +12808,7 @@
         </is>
       </c>
       <c r="H336" s="5" t="n">
-        <v>0.028</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="337">
@@ -12884,7 +12884,7 @@
         </is>
       </c>
       <c r="H338" s="5" t="n">
-        <v>0.006</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="339">
@@ -12922,7 +12922,7 @@
         </is>
       </c>
       <c r="H339" s="5" t="n">
-        <v>0.025</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="340">
@@ -12960,7 +12960,7 @@
         </is>
       </c>
       <c r="H340" s="5" t="n">
-        <v>0.018</v>
+        <v>0.014</v>
       </c>
     </row>
     <row r="341">
@@ -12998,7 +12998,7 @@
         </is>
       </c>
       <c r="H341" s="5" t="n">
-        <v>0.011</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="342">
@@ -13074,7 +13074,7 @@
         </is>
       </c>
       <c r="H343" s="5" t="n">
-        <v>0.017</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="344">
@@ -13112,7 +13112,7 @@
         </is>
       </c>
       <c r="H344" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="345">
@@ -13150,7 +13150,7 @@
         </is>
       </c>
       <c r="H345" s="5" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="346">
@@ -13188,7 +13188,7 @@
         </is>
       </c>
       <c r="H346" s="5" t="n">
-        <v>0.013</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="347">
@@ -13226,7 +13226,7 @@
         </is>
       </c>
       <c r="H347" s="5" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="348">
@@ -13264,7 +13264,7 @@
         </is>
       </c>
       <c r="H348" s="5" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="349">
@@ -13302,7 +13302,7 @@
         </is>
       </c>
       <c r="H349" s="5" t="n">
-        <v>0.008</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="350">
@@ -13378,7 +13378,7 @@
         </is>
       </c>
       <c r="H351" s="5" t="n">
-        <v>0.013</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="352">
@@ -13416,7 +13416,7 @@
         </is>
       </c>
       <c r="H352" s="5" t="n">
-        <v>0.013</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="353">
@@ -13454,7 +13454,7 @@
         </is>
       </c>
       <c r="H353" s="5" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="354">
@@ -13492,7 +13492,7 @@
         </is>
       </c>
       <c r="H354" s="5" t="n">
-        <v>0.017</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="355">
@@ -13530,7 +13530,7 @@
         </is>
       </c>
       <c r="H355" s="5" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="356">
@@ -13568,7 +13568,7 @@
         </is>
       </c>
       <c r="H356" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="357">
@@ -13606,7 +13606,7 @@
         </is>
       </c>
       <c r="H357" s="5" t="n">
-        <v>0.01</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="358">
@@ -13644,7 +13644,7 @@
         </is>
       </c>
       <c r="H358" s="5" t="n">
-        <v>0.002</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="359">
@@ -13682,7 +13682,7 @@
         </is>
       </c>
       <c r="H359" s="5" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="360">
@@ -13720,7 +13720,7 @@
         </is>
       </c>
       <c r="H360" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="361">
@@ -13758,7 +13758,7 @@
         </is>
       </c>
       <c r="H361" s="5" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="362">
@@ -13796,7 +13796,7 @@
         </is>
       </c>
       <c r="H362" s="5" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="363">
@@ -13864,7 +13864,7 @@
         </is>
       </c>
       <c r="H364" s="5" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="365">
@@ -13898,7 +13898,7 @@
         </is>
       </c>
       <c r="H365" s="5" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
     </row>
     <row r="366">
@@ -13932,7 +13932,7 @@
         </is>
       </c>
       <c r="H366" s="5" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="367">
@@ -13966,7 +13966,7 @@
         </is>
       </c>
       <c r="H367" s="5" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="368">
@@ -14000,7 +14000,7 @@
         </is>
       </c>
       <c r="H368" s="5" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="369">
@@ -14034,7 +14034,7 @@
         </is>
       </c>
       <c r="H369" s="5" t="n">
-        <v>0.004</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="370">
@@ -14068,7 +14068,7 @@
         </is>
       </c>
       <c r="H370" s="5" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="371">
@@ -14102,7 +14102,7 @@
         </is>
       </c>
       <c r="H371" s="5" t="n">
-        <v>0.013</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="372">
@@ -14204,7 +14204,7 @@
         </is>
       </c>
       <c r="H374" s="5" t="n">
-        <v>0.016</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="375">
@@ -14276,7 +14276,7 @@
         </is>
       </c>
       <c r="H376" s="5" t="n">
-        <v>0.018</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="377">
@@ -14314,7 +14314,7 @@
         </is>
       </c>
       <c r="H377" s="5" t="n">
-        <v>0.014</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="378">
@@ -14352,7 +14352,7 @@
         </is>
       </c>
       <c r="H378" s="5" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="379">
@@ -14390,7 +14390,7 @@
         </is>
       </c>
       <c r="H379" s="5" t="n">
-        <v>0.004</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="380">
@@ -14428,7 +14428,7 @@
         </is>
       </c>
       <c r="H380" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="381">
@@ -14466,7 +14466,7 @@
         </is>
       </c>
       <c r="H381" s="5" t="n">
-        <v>0.004</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="382">
@@ -14504,7 +14504,7 @@
         </is>
       </c>
       <c r="H382" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="383">
@@ -14542,7 +14542,7 @@
         </is>
       </c>
       <c r="H383" s="5" t="n">
-        <v>0.015</v>
+        <v>0.011</v>
       </c>
     </row>
     <row r="384">
@@ -14580,7 +14580,7 @@
         </is>
       </c>
       <c r="H384" s="5" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="385">
@@ -14618,7 +14618,7 @@
         </is>
       </c>
       <c r="H385" s="5" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="386">
@@ -14656,7 +14656,7 @@
         </is>
       </c>
       <c r="H386" s="5" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="387">
@@ -14694,7 +14694,7 @@
         </is>
       </c>
       <c r="H387" s="5" t="n">
-        <v>0.074</v>
+        <v>0.051</v>
       </c>
     </row>
     <row r="388">
@@ -14732,7 +14732,7 @@
         </is>
       </c>
       <c r="H388" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="389">
@@ -14770,7 +14770,7 @@
         </is>
       </c>
       <c r="H389" s="5" t="n">
-        <v>0.092</v>
+        <v>0.074</v>
       </c>
     </row>
     <row r="390">
@@ -14846,7 +14846,7 @@
         </is>
       </c>
       <c r="H391" s="5" t="n">
-        <v>0.026</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="392">
@@ -14884,7 +14884,7 @@
         </is>
       </c>
       <c r="H392" s="5" t="n">
-        <v>0.014</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="393">
@@ -14922,7 +14922,7 @@
         </is>
       </c>
       <c r="H393" s="5" t="n">
-        <v>0.013</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="394">
@@ -14960,7 +14960,7 @@
         </is>
       </c>
       <c r="H394" s="5" t="n">
-        <v>0.01</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="395">
@@ -14998,7 +14998,7 @@
         </is>
       </c>
       <c r="H395" s="5" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="396">
@@ -15036,7 +15036,7 @@
         </is>
       </c>
       <c r="H396" s="5" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="397">
@@ -15150,7 +15150,7 @@
         </is>
       </c>
       <c r="H399" s="5" t="n">
-        <v>0.021</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="400">
@@ -15188,7 +15188,7 @@
         </is>
       </c>
       <c r="H400" s="5" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="401">
@@ -15226,7 +15226,7 @@
         </is>
       </c>
       <c r="H401" s="5" t="n">
-        <v>0.012</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="402">
@@ -15264,7 +15264,7 @@
         </is>
       </c>
       <c r="H402" s="5" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="403">
@@ -15302,7 +15302,7 @@
         </is>
       </c>
       <c r="H403" s="5" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="404">
@@ -15340,7 +15340,7 @@
         </is>
       </c>
       <c r="H404" s="5" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="405">
@@ -15378,7 +15378,7 @@
         </is>
       </c>
       <c r="H405" s="5" t="n">
-        <v>0.011</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="406">
@@ -15416,7 +15416,7 @@
         </is>
       </c>
       <c r="H406" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="407">
@@ -15454,7 +15454,7 @@
         </is>
       </c>
       <c r="H407" s="5" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="408">
@@ -15530,7 +15530,7 @@
         </is>
       </c>
       <c r="H409" s="5" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="410">
@@ -15568,7 +15568,7 @@
         </is>
       </c>
       <c r="H410" s="5" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="411">
@@ -15644,7 +15644,7 @@
         </is>
       </c>
       <c r="H412" s="5" t="n">
-        <v>0.001</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="413">
@@ -15720,7 +15720,7 @@
         </is>
       </c>
       <c r="H414" s="5" t="n">
-        <v>0.006</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="415">
@@ -15758,7 +15758,7 @@
         </is>
       </c>
       <c r="H415" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="416">
@@ -15796,7 +15796,7 @@
         </is>
       </c>
       <c r="H416" s="5" t="n">
-        <v>0.004</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="417">
@@ -15872,7 +15872,7 @@
         </is>
       </c>
       <c r="H418" s="5" t="n">
-        <v>0.035</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="419">
@@ -15910,7 +15910,7 @@
         </is>
       </c>
       <c r="H419" s="5" t="n">
-        <v>0.003</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="420">
@@ -15948,7 +15948,7 @@
         </is>
       </c>
       <c r="H420" s="5" t="n">
-        <v>0.013</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="421">
@@ -15986,7 +15986,7 @@
         </is>
       </c>
       <c r="H421" s="5" t="n">
-        <v>0.019</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="422">
@@ -16024,7 +16024,7 @@
         </is>
       </c>
       <c r="H422" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="423">
@@ -16062,7 +16062,7 @@
         </is>
       </c>
       <c r="H423" s="5" t="n">
-        <v>0.01</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="424">
@@ -16100,7 +16100,7 @@
         </is>
       </c>
       <c r="H424" s="5" t="n">
-        <v>0.03</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="425">
@@ -16138,7 +16138,7 @@
         </is>
       </c>
       <c r="H425" s="5" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="426">
@@ -16176,7 +16176,7 @@
         </is>
       </c>
       <c r="H426" s="5" t="n">
-        <v>0.006</v>
+        <v>0.003</v>
       </c>
     </row>
     <row r="427">
@@ -16214,7 +16214,7 @@
         </is>
       </c>
       <c r="H427" s="5" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="428">
@@ -16252,7 +16252,7 @@
         </is>
       </c>
       <c r="H428" s="5" t="n">
-        <v>0.028</v>
+        <v>0.022</v>
       </c>
     </row>
     <row r="429">
@@ -16290,7 +16290,7 @@
         </is>
       </c>
       <c r="H429" s="5" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="430">
@@ -16328,7 +16328,7 @@
         </is>
       </c>
       <c r="H430" s="5" t="n">
-        <v>0.016</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="431">
@@ -16366,7 +16366,7 @@
         </is>
       </c>
       <c r="H431" s="5" t="n">
-        <v>0.021</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="432">
@@ -16404,7 +16404,7 @@
         </is>
       </c>
       <c r="H432" s="5" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="433">
@@ -16442,7 +16442,7 @@
         </is>
       </c>
       <c r="H433" s="5" t="n">
-        <v>0.002</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="434">
@@ -16480,7 +16480,7 @@
         </is>
       </c>
       <c r="H434" s="5" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="435">
@@ -16556,7 +16556,7 @@
         </is>
       </c>
       <c r="H436" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="437">
@@ -16594,7 +16594,7 @@
         </is>
       </c>
       <c r="H437" s="5" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="438">
@@ -16632,7 +16632,7 @@
         </is>
       </c>
       <c r="H438" s="5" t="n">
-        <v>0.011</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="439">
@@ -16670,7 +16670,7 @@
         </is>
       </c>
       <c r="H439" s="5" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="440">
@@ -16784,7 +16784,7 @@
         </is>
       </c>
       <c r="H442" s="5" t="n">
-        <v>0.003</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="443">
@@ -16822,7 +16822,7 @@
         </is>
       </c>
       <c r="H443" s="5" t="n">
-        <v>0</v>
+        <v>0.025</v>
       </c>
     </row>
     <row r="444">
@@ -16898,7 +16898,7 @@
         </is>
       </c>
       <c r="H445" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="446">
@@ -16936,7 +16936,7 @@
         </is>
       </c>
       <c r="H446" s="5" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="447">
@@ -17012,7 +17012,7 @@
         </is>
       </c>
       <c r="H448" s="5" t="n">
-        <v>0.008</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="449">
@@ -17050,7 +17050,7 @@
         </is>
       </c>
       <c r="H449" s="5" t="n">
-        <v>0.004</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="450">
@@ -17164,7 +17164,7 @@
         </is>
       </c>
       <c r="H452" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="453">
@@ -17198,7 +17198,7 @@
         </is>
       </c>
       <c r="H453" s="5" t="n">
-        <v>0.03</v>
+        <v>0.021</v>
       </c>
     </row>
     <row r="454">
@@ -17232,7 +17232,7 @@
         </is>
       </c>
       <c r="H454" s="5" t="n">
-        <v>0.019</v>
+        <v>0.013</v>
       </c>
     </row>
     <row r="455">
@@ -17266,7 +17266,7 @@
         </is>
       </c>
       <c r="H455" s="5" t="n">
-        <v>0.028</v>
+        <v>0.018</v>
       </c>
     </row>
     <row r="456">
@@ -17300,7 +17300,7 @@
         </is>
       </c>
       <c r="H456" s="5" t="n">
-        <v>0.012</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="457">
@@ -17334,7 +17334,7 @@
         </is>
       </c>
       <c r="H457" s="5" t="n">
-        <v>0.011</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="458">
@@ -17368,7 +17368,7 @@
         </is>
       </c>
       <c r="H458" s="5" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="459">
@@ -17406,7 +17406,7 @@
         </is>
       </c>
       <c r="H459" s="5" t="n">
-        <v>0.049</v>
+        <v>0.048</v>
       </c>
     </row>
     <row r="460">
@@ -17444,7 +17444,7 @@
         </is>
       </c>
       <c r="H460" s="5" t="n">
-        <v>0.019</v>
+        <v>0.015</v>
       </c>
     </row>
     <row r="461">
@@ -17482,7 +17482,7 @@
         </is>
       </c>
       <c r="H461" s="5" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="462">
@@ -17558,7 +17558,7 @@
         </is>
       </c>
       <c r="H463" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="464">
@@ -17596,7 +17596,7 @@
         </is>
       </c>
       <c r="H464" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="465">
@@ -17672,7 +17672,7 @@
         </is>
       </c>
       <c r="H466" s="5" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="467">
@@ -17710,7 +17710,7 @@
         </is>
       </c>
       <c r="H467" s="5" t="n">
-        <v>0.021</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="468">
@@ -17748,7 +17748,7 @@
         </is>
       </c>
       <c r="H468" s="5" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="469">
@@ -17786,7 +17786,7 @@
         </is>
       </c>
       <c r="H469" s="5" t="n">
-        <v>0.024</v>
+        <v>0.019</v>
       </c>
     </row>
     <row r="470">
@@ -17824,7 +17824,7 @@
         </is>
       </c>
       <c r="H470" s="5" t="n">
-        <v>0.019</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="471">
@@ -17862,7 +17862,7 @@
         </is>
       </c>
       <c r="H471" s="5" t="n">
-        <v>0.021</v>
+        <v>0.017</v>
       </c>
     </row>
     <row r="472">
@@ -17938,7 +17938,7 @@
         </is>
       </c>
       <c r="H473" s="5" t="n">
-        <v>0.011</v>
+        <v>0.008</v>
       </c>
     </row>
     <row r="474">
@@ -18014,7 +18014,7 @@
         </is>
       </c>
       <c r="H475" s="5" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="476">
@@ -18052,7 +18052,7 @@
         </is>
       </c>
       <c r="H476" s="5" t="n">
-        <v>0.015</v>
+        <v>0.012</v>
       </c>
     </row>
     <row r="477">
@@ -18090,7 +18090,7 @@
         </is>
       </c>
       <c r="H477" s="5" t="n">
-        <v>0</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="478">
@@ -18128,7 +18128,7 @@
         </is>
       </c>
       <c r="H478" s="5" t="n">
-        <v>0.013</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="479">
@@ -18204,7 +18204,7 @@
         </is>
       </c>
       <c r="H480" s="5" t="n">
-        <v>0.003</v>
+        <v>0.007</v>
       </c>
     </row>
     <row r="481">
@@ -18242,7 +18242,7 @@
         </is>
       </c>
       <c r="H481" s="5" t="n">
-        <v>0.005</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="482">
@@ -18280,7 +18280,7 @@
         </is>
       </c>
       <c r="H482" s="5" t="n">
-        <v>0.007</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="483">
@@ -18318,7 +18318,7 @@
         </is>
       </c>
       <c r="H483" s="5" t="n">
-        <v>0.013</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="484">
@@ -18356,7 +18356,7 @@
         </is>
       </c>
       <c r="H484" s="5" t="n">
-        <v>0.013</v>
+        <v>0.008999999999999999</v>
       </c>
     </row>
     <row r="485">
@@ -18394,7 +18394,7 @@
         </is>
       </c>
       <c r="H485" s="5" t="n">
-        <v>0.005</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="486">
@@ -18432,7 +18432,7 @@
         </is>
       </c>
       <c r="H486" s="5" t="n">
-        <v>0.004</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="487">
@@ -18470,7 +18470,7 @@
         </is>
       </c>
       <c r="H487" s="5" t="n">
-        <v>0.016</v>
+        <v>0.01</v>
       </c>
     </row>
     <row r="488">
@@ -18508,7 +18508,7 @@
         </is>
       </c>
       <c r="H488" s="5" t="n">
-        <v>0.004</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="489">
@@ -18546,7 +18546,7 @@
         </is>
       </c>
       <c r="H489" s="5" t="n">
-        <v>0.01</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="490">
@@ -18584,7 +18584,7 @@
         </is>
       </c>
       <c r="H490" s="5" t="n">
-        <v>0.001</v>
+        <v>0.006</v>
       </c>
     </row>
     <row r="491">
@@ -18656,7 +18656,7 @@
         </is>
       </c>
       <c r="H492" s="5" t="n">
-        <v>1.583</v>
+        <v>1.736</v>
       </c>
     </row>
     <row r="493">
@@ -18690,7 +18690,7 @@
         </is>
       </c>
       <c r="H493" s="5" t="n">
-        <v>0.228</v>
+        <v>0.234</v>
       </c>
     </row>
     <row r="494">
@@ -18724,7 +18724,7 @@
         </is>
       </c>
       <c r="H494" s="5" t="n">
-        <v>0.186</v>
+        <v>0.205</v>
       </c>
     </row>
     <row r="495">
@@ -18758,7 +18758,7 @@
         </is>
       </c>
       <c r="H495" s="5" t="n">
-        <v>0.128</v>
+        <v>0.146</v>
       </c>
     </row>
     <row r="496">
@@ -18792,7 +18792,7 @@
         </is>
       </c>
       <c r="H496" s="5" t="n">
-        <v>0.138</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="497">
@@ -18826,7 +18826,7 @@
         </is>
       </c>
       <c r="H497" s="5" t="n">
-        <v>0.171</v>
+        <v>0.147</v>
       </c>
     </row>
     <row r="498">
@@ -18860,7 +18860,7 @@
         </is>
       </c>
       <c r="H498" s="5" t="n">
-        <v>0.118</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="499">
@@ -18894,7 +18894,7 @@
         </is>
       </c>
       <c r="H499" s="5" t="n">
-        <v>0.121</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="500">
@@ -18928,7 +18928,7 @@
         </is>
       </c>
       <c r="H500" s="5" t="n">
-        <v>0.156</v>
+        <v>0.168</v>
       </c>
     </row>
     <row r="501">
@@ -18962,7 +18962,7 @@
         </is>
       </c>
       <c r="H501" s="5" t="n">
-        <v>0.22</v>
+        <v>0.194</v>
       </c>
     </row>
     <row r="502">
@@ -18996,7 +18996,7 @@
         </is>
       </c>
       <c r="H502" s="5" t="n">
-        <v>0.25</v>
+        <v>0.183</v>
       </c>
     </row>
     <row r="503">
@@ -19030,7 +19030,7 @@
         </is>
       </c>
       <c r="H503" s="5" t="n">
-        <v>0.053</v>
+        <v>0.042</v>
       </c>
     </row>
     <row r="504">
@@ -19064,7 +19064,7 @@
         </is>
       </c>
       <c r="H504" s="5" t="n">
-        <v>0.14</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="505">
@@ -19098,7 +19098,7 @@
         </is>
       </c>
       <c r="H505" s="5" t="n">
-        <v>0.245</v>
+        <v>0.222</v>
       </c>
     </row>
     <row r="506">
@@ -19132,7 +19132,7 @@
         </is>
       </c>
       <c r="H506" s="5" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.08799999999999999</v>
       </c>
     </row>
     <row r="507">
@@ -19166,7 +19166,7 @@
         </is>
       </c>
       <c r="H507" s="5" t="n">
-        <v>0.032</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="508">
@@ -19200,7 +19200,7 @@
         </is>
       </c>
       <c r="H508" s="5" t="n">
-        <v>0.03</v>
+        <v>0.029</v>
       </c>
     </row>
     <row r="509">
@@ -19234,7 +19234,7 @@
         </is>
       </c>
       <c r="H509" s="5" t="n">
-        <v>0.076</v>
+        <v>0.075</v>
       </c>
     </row>
     <row r="510">
@@ -19268,7 +19268,7 @@
         </is>
       </c>
       <c r="H510" s="5" t="n">
-        <v>0.158</v>
+        <v>0.139</v>
       </c>
     </row>
     <row r="511">
@@ -19302,7 +19302,7 @@
         </is>
       </c>
       <c r="H511" s="5" t="n">
-        <v>0.194</v>
+        <v>0.197</v>
       </c>
     </row>
     <row r="512">
@@ -19336,7 +19336,7 @@
         </is>
       </c>
       <c r="H512" s="5" t="n">
-        <v>0.058</v>
+        <v>0.078</v>
       </c>
     </row>
     <row r="513">
@@ -19370,7 +19370,7 @@
         </is>
       </c>
       <c r="H513" s="5" t="n">
-        <v>0.046</v>
+        <v>0.073</v>
       </c>
     </row>
     <row r="514">
@@ -19404,7 +19404,7 @@
         </is>
       </c>
       <c r="H514" s="5" t="n">
-        <v>0.024</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="515">
@@ -19438,7 +19438,7 @@
         </is>
       </c>
       <c r="H515" s="5" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.081</v>
       </c>
     </row>
     <row r="516">
@@ -19472,7 +19472,7 @@
         </is>
       </c>
       <c r="H516" s="5" t="n">
-        <v>0.046</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="517">
@@ -19506,7 +19506,7 @@
         </is>
       </c>
       <c r="H517" s="5" t="n">
-        <v>0.039</v>
+        <v>0.034</v>
       </c>
     </row>
     <row r="518">
@@ -19540,7 +19540,7 @@
         </is>
       </c>
       <c r="H518" s="5" t="n">
-        <v>0.13</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="519">
@@ -19574,7 +19574,7 @@
         </is>
       </c>
       <c r="H519" s="5" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
     </row>
     <row r="520">
@@ -19642,7 +19642,7 @@
         </is>
       </c>
       <c r="H521" s="5" t="n">
-        <v>0.102</v>
+        <v>0.101</v>
       </c>
     </row>
     <row r="522">
@@ -19676,7 +19676,7 @@
         </is>
       </c>
       <c r="H522" s="5" t="n">
-        <v>0.053</v>
+        <v>0.054</v>
       </c>
     </row>
     <row r="523">
@@ -19710,7 +19710,7 @@
         </is>
       </c>
       <c r="H523" s="5" t="n">
-        <v>0.121</v>
+        <v>0.108</v>
       </c>
     </row>
     <row r="524">
@@ -19744,7 +19744,7 @@
         </is>
       </c>
       <c r="H524" s="5" t="n">
-        <v>0.168</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="525">
@@ -19778,7 +19778,7 @@
         </is>
       </c>
       <c r="H525" s="5" t="n">
-        <v>0.154</v>
+        <v>0.092</v>
       </c>
     </row>
     <row r="526">
@@ -19812,7 +19812,7 @@
         </is>
       </c>
       <c r="H526" s="5" t="n">
-        <v>0.048</v>
+        <v>0.044</v>
       </c>
     </row>
     <row r="527">
@@ -19846,7 +19846,7 @@
         </is>
       </c>
       <c r="H527" s="5" t="n">
-        <v>0.078</v>
+        <v>0.061</v>
       </c>
     </row>
     <row r="528">
@@ -19880,7 +19880,7 @@
         </is>
       </c>
       <c r="H528" s="5" t="n">
-        <v>0.082</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="529">
@@ -19914,7 +19914,7 @@
         </is>
       </c>
       <c r="H529" s="5" t="n">
-        <v>0.078</v>
+        <v>0.077</v>
       </c>
     </row>
     <row r="530">
@@ -19948,7 +19948,7 @@
         </is>
       </c>
       <c r="H530" s="5" t="n">
-        <v>0.061</v>
+        <v>0.052</v>
       </c>
     </row>
     <row r="531">
@@ -19982,7 +19982,7 @@
         </is>
       </c>
       <c r="H531" s="5" t="n">
-        <v>0.594</v>
+        <v>0.526</v>
       </c>
     </row>
     <row r="532">
@@ -20016,7 +20016,7 @@
         </is>
       </c>
       <c r="H532" s="5" t="n">
-        <v>2.904</v>
+        <v>2.953</v>
       </c>
     </row>
     <row r="533">
@@ -20050,7 +20050,7 @@
         </is>
       </c>
       <c r="H533" s="5" t="n">
-        <v>0.029</v>
+        <v>0.053</v>
       </c>
     </row>
     <row r="534">
@@ -20084,7 +20084,7 @@
         </is>
       </c>
       <c r="H534" s="5" t="n">
-        <v>0.17</v>
+        <v>0.161</v>
       </c>
     </row>
     <row r="535">
@@ -20118,7 +20118,7 @@
         </is>
       </c>
       <c r="H535" s="5" t="n">
-        <v>0.261</v>
+        <v>0.308</v>
       </c>
     </row>
     <row r="536">
@@ -20152,7 +20152,7 @@
         </is>
       </c>
       <c r="H536" s="5" t="n">
-        <v>0.126</v>
+        <v>0.153</v>
       </c>
     </row>
     <row r="537">
@@ -20186,7 +20186,7 @@
         </is>
       </c>
       <c r="H537" s="5" t="n">
-        <v>0.109</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="538">
@@ -20220,7 +20220,7 @@
         </is>
       </c>
       <c r="H538" s="5" t="n">
-        <v>0.107</v>
+        <v>0.122</v>
       </c>
     </row>
     <row r="539">
@@ -20254,7 +20254,7 @@
         </is>
       </c>
       <c r="H539" s="5" t="n">
-        <v>0.115</v>
+        <v>0.137</v>
       </c>
     </row>
     <row r="540">
@@ -20288,7 +20288,7 @@
         </is>
       </c>
       <c r="H540" s="5" t="n">
-        <v>0.112</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="541">
@@ -20322,7 +20322,7 @@
         </is>
       </c>
       <c r="H541" s="5" t="n">
-        <v>0.11</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="542">
@@ -20356,7 +20356,7 @@
         </is>
       </c>
       <c r="H542" s="5" t="n">
-        <v>0.097</v>
+        <v>0.106</v>
       </c>
     </row>
     <row r="543">
@@ -20390,7 +20390,7 @@
         </is>
       </c>
       <c r="H543" s="5" t="n">
-        <v>0.152</v>
+        <v>0.187</v>
       </c>
     </row>
     <row r="544">
@@ -20424,7 +20424,7 @@
         </is>
       </c>
       <c r="H544" s="5" t="n">
-        <v>0.191</v>
+        <v>0.223</v>
       </c>
     </row>
     <row r="545">
@@ -20458,7 +20458,7 @@
         </is>
       </c>
       <c r="H545" s="5" t="n">
-        <v>0.11</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="546">
@@ -20492,7 +20492,7 @@
         </is>
       </c>
       <c r="H546" s="5" t="n">
-        <v>0.089</v>
+        <v>0.099</v>
       </c>
     </row>
     <row r="547">
@@ -20526,7 +20526,7 @@
         </is>
       </c>
       <c r="H547" s="5" t="n">
-        <v>0.106</v>
+        <v>0.118</v>
       </c>
     </row>
     <row r="548">
@@ -20560,7 +20560,7 @@
         </is>
       </c>
       <c r="H548" s="5" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.08599999999999999</v>
       </c>
     </row>
     <row r="549">
@@ -20594,7 +20594,7 @@
         </is>
       </c>
       <c r="H549" s="5" t="n">
-        <v>0.101</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="550">
@@ -20628,7 +20628,7 @@
         </is>
       </c>
       <c r="H550" s="5" t="n">
-        <v>0.107</v>
+        <v>0.105</v>
       </c>
     </row>
     <row r="551">
@@ -20662,7 +20662,7 @@
         </is>
       </c>
       <c r="H551" s="5" t="n">
-        <v>0.121</v>
+        <v>0.117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>